<commit_message>
experiment gebouwd nog niet correct
</commit_message>
<xml_diff>
--- a/PaintShop Beste Schema 4M.xlsx
+++ b/PaintShop Beste Schema 4M.xlsx
@@ -488,7 +488,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ORD01</t>
+          <t>ORD02</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -506,19 +506,19 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>7.142857142857143</v>
+        <v>9.523809523809524</v>
       </c>
       <c r="G2" t="n">
-        <v>7.142857142857143</v>
+        <v>9.523809523809524</v>
       </c>
       <c r="H2" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -527,7 +527,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ORD11</t>
+          <t>ORD01</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -539,34 +539,34 @@
         <v>2</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
+        <v>12.52380952380952</v>
+      </c>
+      <c r="F3" t="n">
         <v>7.142857142857143</v>
       </c>
-      <c r="F3" t="n">
-        <v>10.95238095238095</v>
-      </c>
       <c r="G3" t="n">
-        <v>18.09523809523809</v>
+        <v>19.66666666666667</v>
       </c>
       <c r="H3" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1.666666666666668</v>
       </c>
       <c r="J3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>16.66666666666668</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ORD12</t>
+          <t>ORD11</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -578,34 +578,34 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>22.09523809523809</v>
+        <v>19.66666666666667</v>
       </c>
       <c r="F4" t="n">
-        <v>10.47619047619048</v>
+        <v>10.95238095238095</v>
       </c>
       <c r="G4" t="n">
-        <v>32.57142857142857</v>
+        <v>30.61904761904762</v>
       </c>
       <c r="H4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I4" t="n">
-        <v>14.57142857142857</v>
+        <v>10.61904761904762</v>
       </c>
       <c r="J4" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="K4" t="n">
-        <v>87.42857142857142</v>
+        <v>127.4285714285714</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ORD43</t>
+          <t>ORD25</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -620,22 +620,22 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>32.57142857142857</v>
+        <v>30.61904761904762</v>
       </c>
       <c r="F5" t="n">
-        <v>5.714285714285714</v>
+        <v>10</v>
       </c>
       <c r="G5" t="n">
-        <v>38.28571428571428</v>
+        <v>40.61904761904762</v>
       </c>
       <c r="H5" t="n">
-        <v>78</v>
+        <v>53</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -644,7 +644,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ORD10</t>
+          <t>ORD39</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -656,34 +656,34 @@
         <v>5</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E6" t="n">
-        <v>38.28571428571428</v>
+        <v>47.61904761904762</v>
       </c>
       <c r="F6" t="n">
-        <v>5.714285714285714</v>
+        <v>8.571428571428571</v>
       </c>
       <c r="G6" t="n">
-        <v>44</v>
+        <v>56.19047619047619</v>
       </c>
       <c r="H6" t="n">
-        <v>41</v>
+        <v>99</v>
       </c>
       <c r="I6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J6" t="n">
         <v>9</v>
       </c>
       <c r="K6" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ORD35</t>
+          <t>ORD42</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -698,22 +698,22 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>44</v>
+        <v>56.19047619047619</v>
       </c>
       <c r="F7" t="n">
-        <v>5.714285714285714</v>
+        <v>10.47619047619048</v>
       </c>
       <c r="G7" t="n">
-        <v>49.71428571428572</v>
+        <v>66.66666666666667</v>
       </c>
       <c r="H7" t="n">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -722,7 +722,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ORD16</t>
+          <t>ORD17</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -734,25 +734,25 @@
         <v>7</v>
       </c>
       <c r="D8" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>54.71428571428572</v>
+        <v>66.66666666666667</v>
       </c>
       <c r="F8" t="n">
-        <v>7.619047619047619</v>
+        <v>6.666666666666667</v>
       </c>
       <c r="G8" t="n">
-        <v>62.33333333333334</v>
+        <v>73.33333333333334</v>
       </c>
       <c r="H8" t="n">
-        <v>63</v>
+        <v>85</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -761,7 +761,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ORD18</t>
+          <t>ORD28</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -773,34 +773,34 @@
         <v>8</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E9" t="n">
-        <v>62.33333333333334</v>
+        <v>75.33333333333334</v>
       </c>
       <c r="F9" t="n">
-        <v>10</v>
+        <v>10.95238095238095</v>
       </c>
       <c r="G9" t="n">
-        <v>72.33333333333334</v>
+        <v>86.28571428571429</v>
       </c>
       <c r="H9" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>4.285714285714292</v>
       </c>
       <c r="J9" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>25.71428571428575</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ORD34</t>
+          <t>ORD31</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -812,34 +812,34 @@
         <v>9</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>72.33333333333334</v>
+        <v>88.28571428571429</v>
       </c>
       <c r="F10" t="n">
-        <v>10.47619047619048</v>
+        <v>8.571428571428571</v>
       </c>
       <c r="G10" t="n">
-        <v>82.80952380952382</v>
+        <v>96.85714285714286</v>
       </c>
       <c r="H10" t="n">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="I10" t="n">
-        <v>2.809523809523824</v>
+        <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="K10" t="n">
-        <v>30.90476190476207</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ORD31</t>
+          <t>ORD24</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -854,22 +854,22 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>82.80952380952382</v>
+        <v>96.85714285714286</v>
       </c>
       <c r="F11" t="n">
-        <v>8.571428571428571</v>
+        <v>9.047619047619047</v>
       </c>
       <c r="G11" t="n">
-        <v>91.38095238095239</v>
+        <v>105.9047619047619</v>
       </c>
       <c r="H11" t="n">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="I11" t="n">
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -878,7 +878,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ORD24</t>
+          <t>ORD37</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -893,31 +893,31 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>91.38095238095239</v>
+        <v>105.9047619047619</v>
       </c>
       <c r="F12" t="n">
-        <v>9.047619047619047</v>
+        <v>5.238095238095238</v>
       </c>
       <c r="G12" t="n">
-        <v>100.4285714285714</v>
+        <v>111.1428571428572</v>
       </c>
       <c r="H12" t="n">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>1.142857142857153</v>
       </c>
       <c r="J12" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>10.28571428571438</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ORD38</t>
+          <t>ORD44</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -929,34 +929,34 @@
         <v>12</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>105.4285714285714</v>
+        <v>111.1428571428572</v>
       </c>
       <c r="F13" t="n">
-        <v>11.42857142857143</v>
+        <v>10.95238095238095</v>
       </c>
       <c r="G13" t="n">
-        <v>116.8571428571429</v>
+        <v>122.0952380952381</v>
       </c>
       <c r="H13" t="n">
-        <v>115</v>
+        <v>82</v>
       </c>
       <c r="I13" t="n">
-        <v>1.857142857142875</v>
+        <v>40.0952380952381</v>
       </c>
       <c r="J13" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="K13" t="n">
-        <v>24.14285714285738</v>
+        <v>240.5714285714286</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ORD05</t>
+          <t>ORD03</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -974,19 +974,19 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>6.190476190476191</v>
+        <v>8.571428571428571</v>
       </c>
       <c r="G14" t="n">
-        <v>6.190476190476191</v>
+        <v>8.571428571428571</v>
       </c>
       <c r="H14" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -995,7 +995,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ORD02</t>
+          <t>ORD04</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1007,34 +1007,34 @@
         <v>2</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>8.19047619047619</v>
+        <v>8.571428571428571</v>
       </c>
       <c r="F15" t="n">
-        <v>9.523809523809524</v>
+        <v>8.095238095238095</v>
       </c>
       <c r="G15" t="n">
-        <v>17.71428571428572</v>
+        <v>16.66666666666666</v>
       </c>
       <c r="H15" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>1.666666666666664</v>
       </c>
       <c r="J15" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>24.99999999999996</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ORD14</t>
+          <t>ORD10</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1049,22 +1049,22 @@
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>17.71428571428572</v>
+        <v>16.66666666666666</v>
       </c>
       <c r="F16" t="n">
-        <v>11.90476190476191</v>
+        <v>5.714285714285714</v>
       </c>
       <c r="G16" t="n">
-        <v>29.61904761904762</v>
+        <v>22.38095238095238</v>
       </c>
       <c r="H16" t="n">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -1073,7 +1073,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ORD33</t>
+          <t>ORD12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1088,25 +1088,25 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>29.61904761904762</v>
+        <v>22.38095238095238</v>
       </c>
       <c r="F17" t="n">
-        <v>10</v>
+        <v>10.47619047619048</v>
       </c>
       <c r="G17" t="n">
-        <v>39.61904761904762</v>
+        <v>32.85714285714285</v>
       </c>
       <c r="H17" t="n">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>14.85714285714285</v>
       </c>
       <c r="J17" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>89.14285714285712</v>
       </c>
     </row>
     <row r="18">
@@ -1124,16 +1124,16 @@
         <v>5</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E18" t="n">
-        <v>39.61904761904762</v>
+        <v>41.85714285714285</v>
       </c>
       <c r="F18" t="n">
         <v>10</v>
       </c>
       <c r="G18" t="n">
-        <v>49.61904761904762</v>
+        <v>51.85714285714285</v>
       </c>
       <c r="H18" t="n">
         <v>53</v>
@@ -1166,13 +1166,13 @@
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>49.61904761904762</v>
+        <v>51.85714285714285</v>
       </c>
       <c r="F19" t="n">
         <v>7.142857142857143</v>
       </c>
       <c r="G19" t="n">
-        <v>56.76190476190477</v>
+        <v>59</v>
       </c>
       <c r="H19" t="n">
         <v>61</v>
@@ -1190,7 +1190,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ORD15</t>
+          <t>ORD16</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1202,34 +1202,34 @@
         <v>7</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
-        <v>56.76190476190477</v>
+        <v>61</v>
       </c>
       <c r="F20" t="n">
-        <v>11.42857142857143</v>
+        <v>7.619047619047619</v>
       </c>
       <c r="G20" t="n">
-        <v>68.19047619047619</v>
+        <v>68.61904761904762</v>
       </c>
       <c r="H20" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="I20" t="n">
-        <v>2.19047619047619</v>
+        <v>5.61904761904762</v>
       </c>
       <c r="J20" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K20" t="n">
-        <v>19.71428571428571</v>
+        <v>44.95238095238096</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ORD19</t>
+          <t>ORD27</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1244,31 +1244,31 @@
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>68.19047619047619</v>
+        <v>68.61904761904762</v>
       </c>
       <c r="F21" t="n">
-        <v>9.523809523809524</v>
+        <v>5.714285714285714</v>
       </c>
       <c r="G21" t="n">
-        <v>77.71428571428571</v>
+        <v>74.33333333333333</v>
       </c>
       <c r="H21" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I21" t="n">
-        <v>1.714285714285708</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="K21" t="n">
-        <v>25.71428571428562</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ORD28</t>
+          <t>ORD22</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1280,34 +1280,34 @@
         <v>9</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E22" t="n">
-        <v>77.71428571428571</v>
+        <v>79.33333333333333</v>
       </c>
       <c r="F22" t="n">
-        <v>10.95238095238095</v>
+        <v>6.190476190476191</v>
       </c>
       <c r="G22" t="n">
-        <v>88.66666666666666</v>
+        <v>85.52380952380952</v>
       </c>
       <c r="H22" t="n">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="I22" t="n">
-        <v>6.666666666666657</v>
+        <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="K22" t="n">
-        <v>39.99999999999994</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ORD23</t>
+          <t>ORD26</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1322,31 +1322,31 @@
         <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>88.66666666666666</v>
+        <v>85.52380952380952</v>
       </c>
       <c r="F23" t="n">
-        <v>8.571428571428571</v>
+        <v>10.47619047619048</v>
       </c>
       <c r="G23" t="n">
-        <v>97.23809523809523</v>
+        <v>96</v>
       </c>
       <c r="H23" t="n">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J23" t="n">
         <v>9</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>135</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ORD32</t>
+          <t>ORD38</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1361,31 +1361,31 @@
         <v>0</v>
       </c>
       <c r="E24" t="n">
-        <v>97.23809523809523</v>
+        <v>96</v>
       </c>
       <c r="F24" t="n">
-        <v>9.047619047619047</v>
+        <v>11.42857142857143</v>
       </c>
       <c r="G24" t="n">
-        <v>106.2857142857143</v>
+        <v>107.4285714285714</v>
       </c>
       <c r="H24" t="n">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="I24" t="n">
-        <v>0.2857142857142776</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K24" t="n">
-        <v>3.428571428571331</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ORD30</t>
+          <t>ORD36</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1397,34 +1397,34 @@
         <v>12</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>106.2857142857143</v>
+        <v>110.4285714285714</v>
       </c>
       <c r="F25" t="n">
-        <v>11.42857142857143</v>
+        <v>10.95238095238095</v>
       </c>
       <c r="G25" t="n">
-        <v>117.7142857142857</v>
+        <v>121.3809523809524</v>
       </c>
       <c r="H25" t="n">
-        <v>115</v>
+        <v>82</v>
       </c>
       <c r="I25" t="n">
-        <v>2.714285714285708</v>
+        <v>39.38095238095238</v>
       </c>
       <c r="J25" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="K25" t="n">
-        <v>35.28571428571421</v>
+        <v>236.2857142857143</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ORD04</t>
+          <t>ORD13</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1442,19 +1442,19 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>9.444444444444445</v>
+        <v>6.111111111111111</v>
       </c>
       <c r="G26" t="n">
-        <v>9.444444444444445</v>
+        <v>6.111111111111111</v>
       </c>
       <c r="H26" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -1463,7 +1463,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ORD03</t>
+          <t>ORD21</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1478,31 +1478,31 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
+        <v>6.111111111111111</v>
+      </c>
+      <c r="F27" t="n">
         <v>9.444444444444445</v>
       </c>
-      <c r="F27" t="n">
-        <v>10</v>
-      </c>
       <c r="G27" t="n">
-        <v>19.44444444444444</v>
+        <v>15.55555555555556</v>
       </c>
       <c r="H27" t="n">
-        <v>12</v>
+        <v>69</v>
       </c>
       <c r="I27" t="n">
-        <v>7.444444444444443</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K27" t="n">
-        <v>59.55555555555554</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ORD07</t>
+          <t>ORD05</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1514,34 +1514,34 @@
         <v>3</v>
       </c>
       <c r="D28" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>29.44444444444444</v>
+        <v>15.55555555555556</v>
       </c>
       <c r="F28" t="n">
-        <v>7.777777777777778</v>
+        <v>7.222222222222222</v>
       </c>
       <c r="G28" t="n">
-        <v>37.22222222222222</v>
+        <v>22.77777777777778</v>
       </c>
       <c r="H28" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="I28" t="n">
-        <v>2.222222222222221</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="K28" t="n">
-        <v>31.1111111111111</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ORD13</t>
+          <t>ORD07</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1556,22 +1556,22 @@
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>37.22222222222222</v>
+        <v>22.77777777777778</v>
       </c>
       <c r="F29" t="n">
-        <v>6.111111111111111</v>
+        <v>7.777777777777778</v>
       </c>
       <c r="G29" t="n">
-        <v>43.33333333333333</v>
+        <v>30.55555555555556</v>
       </c>
       <c r="H29" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="I29" t="n">
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
@@ -1580,7 +1580,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ORD21</t>
+          <t>ORD14</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1592,25 +1592,25 @@
         <v>5</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E30" t="n">
-        <v>43.33333333333333</v>
+        <v>32.55555555555556</v>
       </c>
       <c r="F30" t="n">
-        <v>9.444444444444445</v>
+        <v>13.88888888888889</v>
       </c>
       <c r="G30" t="n">
-        <v>52.77777777777777</v>
+        <v>46.44444444444444</v>
       </c>
       <c r="H30" t="n">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -1619,7 +1619,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ORD42</t>
+          <t>ORD15</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1634,22 +1634,22 @@
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>52.77777777777777</v>
+        <v>46.44444444444444</v>
       </c>
       <c r="F31" t="n">
-        <v>12.22222222222222</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="G31" t="n">
-        <v>65</v>
+        <v>59.77777777777778</v>
       </c>
       <c r="H31" t="n">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="I31" t="n">
         <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -1658,7 +1658,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ORD17</t>
+          <t>ORD19</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1673,22 +1673,22 @@
         <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>65</v>
+        <v>59.77777777777778</v>
       </c>
       <c r="F32" t="n">
-        <v>7.777777777777778</v>
+        <v>11.11111111111111</v>
       </c>
       <c r="G32" t="n">
-        <v>72.77777777777777</v>
+        <v>70.88888888888889</v>
       </c>
       <c r="H32" t="n">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="I32" t="n">
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -1697,7 +1697,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ORD36</t>
+          <t>ORD43</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1712,31 +1712,31 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>73.77777777777777</v>
+        <v>71.88888888888889</v>
       </c>
       <c r="F33" t="n">
-        <v>12.77777777777778</v>
+        <v>6.666666666666667</v>
       </c>
       <c r="G33" t="n">
-        <v>86.55555555555554</v>
+        <v>78.55555555555556</v>
       </c>
       <c r="H33" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="I33" t="n">
-        <v>4.555555555555543</v>
+        <v>0.5555555555555571</v>
       </c>
       <c r="J33" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K33" t="n">
-        <v>27.33333333333326</v>
+        <v>4.444444444444457</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ORD40</t>
+          <t>ORD35</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1748,64 +1748,64 @@
         <v>9</v>
       </c>
       <c r="D34" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>91.55555555555554</v>
+        <v>78.55555555555556</v>
       </c>
       <c r="F34" t="n">
-        <v>10.55555555555556</v>
+        <v>6.666666666666667</v>
       </c>
       <c r="G34" t="n">
-        <v>102.1111111111111</v>
+        <v>85.22222222222223</v>
       </c>
       <c r="H34" t="n">
-        <v>106</v>
+        <v>78</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
+        <v>7.222222222222229</v>
       </c>
       <c r="J34" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>57.77777777777783</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ORD06</t>
+          <t>ORD40</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E35" t="n">
-        <v>0</v>
+        <v>92.22222222222223</v>
       </c>
       <c r="F35" t="n">
-        <v>8.888888888888889</v>
+        <v>10.55555555555556</v>
       </c>
       <c r="G35" t="n">
-        <v>8.888888888888889</v>
+        <v>102.7777777777778</v>
       </c>
       <c r="H35" t="n">
-        <v>33</v>
+        <v>106</v>
       </c>
       <c r="I35" t="n">
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
@@ -1814,37 +1814,37 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ORD27</t>
+          <t>ORD45</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
       </c>
       <c r="E36" t="n">
-        <v>8.888888888888889</v>
+        <v>102.7777777777778</v>
       </c>
       <c r="F36" t="n">
-        <v>6.666666666666667</v>
+        <v>6.111111111111111</v>
       </c>
       <c r="G36" t="n">
-        <v>15.55555555555556</v>
+        <v>108.8888888888889</v>
       </c>
       <c r="H36" t="n">
-        <v>78</v>
+        <v>110</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -1853,46 +1853,46 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ORD09</t>
+          <t>ORD29</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>M4</t>
+          <t>M3</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E37" t="n">
-        <v>15.55555555555556</v>
+        <v>113.8888888888889</v>
       </c>
       <c r="F37" t="n">
-        <v>10.55555555555556</v>
+        <v>6.111111111111111</v>
       </c>
       <c r="G37" t="n">
-        <v>26.11111111111111</v>
+        <v>120</v>
       </c>
       <c r="H37" t="n">
-        <v>32</v>
+        <v>110</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>10.00000000000001</v>
       </c>
       <c r="J37" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>90.00000000000013</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ORD08</t>
+          <t>ORD09</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1901,28 +1901,28 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
       </c>
       <c r="E38" t="n">
-        <v>26.11111111111111</v>
+        <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>11.66666666666667</v>
+        <v>10.55555555555556</v>
       </c>
       <c r="G38" t="n">
-        <v>37.77777777777778</v>
+        <v>10.55555555555556</v>
       </c>
       <c r="H38" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
@@ -1931,7 +1931,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ORD25</t>
+          <t>ORD06</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1940,37 +1940,37 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D39" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>42.77777777777778</v>
+        <v>10.55555555555556</v>
       </c>
       <c r="F39" t="n">
-        <v>11.66666666666667</v>
+        <v>8.888888888888889</v>
       </c>
       <c r="G39" t="n">
-        <v>54.44444444444444</v>
+        <v>19.44444444444444</v>
       </c>
       <c r="H39" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="I39" t="n">
-        <v>1.444444444444443</v>
+        <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="K39" t="n">
-        <v>21.66666666666664</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ORD22</t>
+          <t>ORD08</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1979,28 +1979,28 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
       </c>
       <c r="E40" t="n">
-        <v>54.44444444444444</v>
+        <v>19.44444444444444</v>
       </c>
       <c r="F40" t="n">
-        <v>7.222222222222222</v>
+        <v>11.66666666666667</v>
       </c>
       <c r="G40" t="n">
-        <v>61.66666666666666</v>
+        <v>31.11111111111111</v>
       </c>
       <c r="H40" t="n">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="I40" t="n">
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
@@ -2009,7 +2009,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ORD26</t>
+          <t>ORD33</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2018,28 +2018,28 @@
         </is>
       </c>
       <c r="C41" t="n">
+        <v>4</v>
+      </c>
+      <c r="D41" t="n">
         <v>7</v>
       </c>
-      <c r="D41" t="n">
-        <v>0</v>
-      </c>
       <c r="E41" t="n">
-        <v>61.66666666666666</v>
+        <v>38.11111111111111</v>
       </c>
       <c r="F41" t="n">
-        <v>12.22222222222222</v>
+        <v>11.66666666666667</v>
       </c>
       <c r="G41" t="n">
-        <v>73.88888888888889</v>
+        <v>49.77777777777777</v>
       </c>
       <c r="H41" t="n">
-        <v>81</v>
+        <v>53</v>
       </c>
       <c r="I41" t="n">
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
@@ -2048,7 +2048,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ORD45</t>
+          <t>ORD34</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2057,28 +2057,28 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E42" t="n">
-        <v>73.88888888888889</v>
+        <v>51.77777777777777</v>
       </c>
       <c r="F42" t="n">
-        <v>6.111111111111111</v>
+        <v>12.22222222222222</v>
       </c>
       <c r="G42" t="n">
+        <v>63.99999999999999</v>
+      </c>
+      <c r="H42" t="n">
         <v>80</v>
       </c>
-      <c r="H42" t="n">
-        <v>110</v>
-      </c>
       <c r="I42" t="n">
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -2087,7 +2087,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ORD39</t>
+          <t>ORD18</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2096,28 +2096,28 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D43" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>87</v>
+        <v>63.99999999999999</v>
       </c>
       <c r="F43" t="n">
+        <v>11.66666666666667</v>
+      </c>
+      <c r="G43" t="n">
+        <v>75.66666666666666</v>
+      </c>
+      <c r="H43" t="n">
+        <v>78</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" t="n">
         <v>10</v>
-      </c>
-      <c r="G43" t="n">
-        <v>97</v>
-      </c>
-      <c r="H43" t="n">
-        <v>99</v>
-      </c>
-      <c r="I43" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" t="n">
-        <v>9</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>
@@ -2126,7 +2126,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ORD29</t>
+          <t>ORD23</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2135,22 +2135,22 @@
         </is>
       </c>
       <c r="C44" t="n">
+        <v>7</v>
+      </c>
+      <c r="D44" t="n">
+        <v>7</v>
+      </c>
+      <c r="E44" t="n">
+        <v>82.66666666666666</v>
+      </c>
+      <c r="F44" t="n">
         <v>10</v>
       </c>
-      <c r="D44" t="n">
-        <v>2</v>
-      </c>
-      <c r="E44" t="n">
+      <c r="G44" t="n">
+        <v>92.66666666666666</v>
+      </c>
+      <c r="H44" t="n">
         <v>99</v>
-      </c>
-      <c r="F44" t="n">
-        <v>6.111111111111111</v>
-      </c>
-      <c r="G44" t="n">
-        <v>105.1111111111111</v>
-      </c>
-      <c r="H44" t="n">
-        <v>110</v>
       </c>
       <c r="I44" t="n">
         <v>0</v>
@@ -2165,7 +2165,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ORD37</t>
+          <t>ORD32</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2174,37 +2174,37 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D45" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E45" t="n">
-        <v>107.1111111111111</v>
+        <v>92.66666666666666</v>
       </c>
       <c r="F45" t="n">
-        <v>6.111111111111111</v>
+        <v>10.55555555555556</v>
       </c>
       <c r="G45" t="n">
-        <v>113.2222222222222</v>
+        <v>103.2222222222222</v>
       </c>
       <c r="H45" t="n">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="I45" t="n">
-        <v>3.222222222222229</v>
+        <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="K45" t="n">
-        <v>29.00000000000006</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ORD44</t>
+          <t>ORD30</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2213,31 +2213,31 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D46" t="n">
         <v>0</v>
       </c>
       <c r="E46" t="n">
-        <v>113.2222222222222</v>
+        <v>103.2222222222222</v>
       </c>
       <c r="F46" t="n">
-        <v>12.77777777777778</v>
+        <v>13.33333333333333</v>
       </c>
       <c r="G46" t="n">
-        <v>126</v>
+        <v>116.5555555555555</v>
       </c>
       <c r="H46" t="n">
-        <v>82</v>
+        <v>115</v>
       </c>
       <c r="I46" t="n">
-        <v>44</v>
+        <v>1.555555555555543</v>
       </c>
       <c r="J46" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="K46" t="n">
-        <v>264</v>
+        <v>20.22222222222206</v>
       </c>
     </row>
   </sheetData>

</xml_diff>